<commit_message>
Update job tracker 2026-08-06 19:44 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +62,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -467,6 +474,32 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>European Southern Observatory</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Sustainability Procurement Advisor</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>...are located in Garching, near Munich, Germany. At Paranal, ESO ope...</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://recruitment.eso.org/jobs/2026_0041</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-06 20:42 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +62,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -467,6 +474,66 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Associate Sustainability Specialist (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2644410</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>(Senior) Product Sustainability Specialist (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2698687</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-07 05:41 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -475,60 +475,60 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Tanso</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Associate Sustainability Specialist (f/m/x)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://tanso.jobs.personio.de/job/2644410</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Tanso</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>(Senior) Product Sustainability Specialist (f/m/x)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://tanso.jobs.personio.de/job/2698687</t>
         </is>

</xml_diff>

<commit_message>
Update job tracker 2026-08-07 06:29 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -30,7 +30,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -41,6 +41,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
   </fills>
@@ -56,9 +62,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -467,6 +474,144 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent_in (m/w/d) Start-up Intelligence Circular Economy</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>München Kreativquartier</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2723225</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Associate Sustainability Specialist (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2644410</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CSR Jobs in München</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>CSR Jobs in München | NachhaltigeJobs Nachhaltige...</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/csr-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nachhaltigkeit</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/nachhaltigkeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München | NachhaltigeJobs Nachhaltige...</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/umwelt-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-11 13:25 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -475,140 +475,163 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Werkstudent_in (m/w/d) Start-up Intelligence Circular Economy</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>München Kreativquartier</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2723225</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Tanso</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Associate Sustainability Specialist (f/m/x)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://tanso.jobs.personio.de/job/2644410</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>NachhaltigeJobs.de (Munich)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>CSR Jobs in München</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>CSR Jobs in München | NachhaltigeJobs Nachhaltige...</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://www.nachhaltigejobs.de/csr-jobs/muenchen</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Michael Page Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Nachhaltigkeit</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://www.michaelpage.de/jobs/nachhaltigkeit</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>NachhaltigeJobs.de (Munich)</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Umwelt Jobs in München</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Umwelt Jobs in München | NachhaltigeJobs Nachhaltige...</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://www.nachhaltigejobs.de/umwelt-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>BUND Naturschutz in Bayern</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Referent*in für Klimaschutz und Energie (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/referentin-fuer-klimaschutz-und-energie-m/w/d</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update job tracker 2026-08-11 15:16 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +43,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
+        <bgColor rgb="00FDE68A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,9 +76,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -469,6 +490,196 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-22</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent_in (m/w/d) Start-up Intelligence Circular Economy</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>München Kreativquartier</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2723225</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Associate Sustainability Specialist (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2644410</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>CSR Jobs in München</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>CSR Jobs in München | NachhaltigeJobs Nachhaltige...</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/csr-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Nachhaltigkeit</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/nachhaltigkeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>BUND Naturschutz in Bayern</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Referent*in für Klimaschutz und Energie (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/referentin-fuer-klimaschutz-und-energie-m/w/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München | NachhaltigeJobs Nachhaltige...</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/umwelt-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Munich, all roles)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Werkstudent (m/w/d) im Bereich Nachhaltigkeit</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>...im Bereich Nachhaltigkeit in München | Randstad randstad Jobsuche...</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/werkstudent-mwd-im-bereich-nachhaltigkeit_muenchen_c01304109/</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -480,7 +691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -523,6 +734,716 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Assistant to the executive Board (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Garching</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2706851</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Community Manager (m/w/d) - Front Desk MakerSpace Garching</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Garching</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2709394</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Export (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>...rbeiter Export (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-export-wmd/06640-0013462604-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013475955-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-sachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Call Center Agent</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-dienstleistung-und-service/j-call-center-agent/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Buchhaltung</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-finanz-und-rechnungswesen/t-rechnungswesen/j-sachbearbeiter-buchhaltung/</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Auftragssachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-marketing-und-vertrieb/t-vertrieb-und-verkauf/j-auftragssachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz der Geschäftsführung</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz-der-geschaeftsfuehrung/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Bürokaufmann</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-buerokaufmann/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Empfangsmitarbeiter</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-empfangsmitarbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Personalsachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-personalwesen/j-personalsachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Projektassistenz</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-projektassistenz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-sachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Verwaltungsfachangestellter</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-verwaltungsfachangestellter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013471891-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Munich, all roles)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Management-Assistenz (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>...nagement-Assistenz (m/w/d) in München | Randstad randstad Jobsuche...</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/management-assistenz-mwd_muenchen_c01310721/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Facility Management</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/facility-management</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Sales Support &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/sales-support-customer-service</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Amadeus Fire (Munich)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Backoffice</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>...e Köln Leipzig Mainz Mannheim München Münster Nürnberg Stuttgart Fa...</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>https://karriere.amadeus-fire.de/backoffice</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz des Gesamtbetriebsrats ( w/m/d)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>...tbetriebsrats ( w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/assistenz-des-gesamtbetriebsrats-wmd/06604-0013483434-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013482368-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013479384-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Sekretär der Führungsebene (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>...Führungsebene (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sekretär-der-führungsebene-wmd/06604-0013471824-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Kreditsachbearbeiter (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>...sachbearbeiter (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/kreditsachbearbeiter-wmd/06644-0013484134-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Technische Vertriebsassistenz (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>...riebsassistenz (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/technische-vertriebsassistenz-wmd/06604-0013485530-dede</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -534,7 +1455,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,6 +1498,448 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>5 C CarbonPlan 1 job 118</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/carbonplan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>6 F FirstCarbon Solutions (FCS), an ADEC Innovation 1 job 113</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/firstcarbon-solutions-fcs-an-adec-innovation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Sustainability</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Sustainability</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>ESG &amp; Carbon</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/esg-reporting-carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Climate Policy</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/advocacy-policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2 C Climate Collective Foundation 1 job 320</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climate-collective-foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>3 C Climate Action Reserve 2 jobs 164</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climateactionreserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>4 G goodcarbon 3 jobs 127</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/goodcarbon-earth</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>7 C ClimateWorks Foundation 2 jobs 109</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climateworks</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Carbon Capture and Storage (15)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/carbon_capture_and_storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Climate and Energy Analyst (27)</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/climate_and_energy_analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=inline&amp;utm_campaign=upgrade&amp;utm_content=homepage-how-it-works</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F16" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=faq&amp;utm_campaign=upgrade&amp;utm_content=homepage-faq-locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs Newsletter</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F17" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=footer&amp;utm_campaign=upgrade&amp;utm_content=footer</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr"/>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>Why climate.jobs?</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E18" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F18" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/why-climate-jobs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-15 11:15 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -491,190 +491,185 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-07-22</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Werkstudent_in (m/w/d) Start-up Intelligence Circular Economy</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>München Kreativquartier</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2723225</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>Tanso</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Associate Sustainability Specialist (f/m/x)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://tanso.jobs.personio.de/job/2644410</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>NachhaltigeJobs.de (Munich)</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>CSR Jobs in München</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n">
+      <c r="D4" t="n">
         <v>3</v>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>CSR Jobs in München | NachhaltigeJobs Nachhaltige...</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://www.nachhaltigejobs.de/csr-jobs/muenchen</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr"/>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Michael Page Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Nachhaltigkeit</t>
         </is>
       </c>
-      <c r="D5" s="2" t="n">
+      <c r="D5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="2" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
         </is>
       </c>
-      <c r="F5" s="2" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://www.michaelpage.de/jobs/nachhaltigkeit</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>BUND Naturschutz in Bayern</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Referent*in für Klimaschutz und Energie (m/w/d)</t>
         </is>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" t="n">
         <v>1</v>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/referentin-fuer-klimaschutz-und-energie-m/w/d</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
-      <c r="B7" s="2" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>NachhaltigeJobs.de (Munich)</t>
         </is>
       </c>
-      <c r="C7" s="2" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Umwelt Jobs in München</t>
         </is>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="2" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Umwelt Jobs in München | NachhaltigeJobs Nachhaltige...</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://www.nachhaltigejobs.de/umwelt-jobs/muenchen</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr"/>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Randstad Germany (Munich, all roles)</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Werkstudent (m/w/d) im Bereich Nachhaltigkeit</t>
         </is>
       </c>
-      <c r="D8" s="2" t="n">
+      <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>...im Bereich Nachhaltigkeit in München | Randstad randstad Jobsuche...</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/werkstudent-mwd-im-bereich-nachhaltigkeit_muenchen_c01304109/</t>
         </is>
@@ -691,7 +686,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -737,138 +732,140 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Planet A Foods</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Office Management &amp; HR - Werkstudent (f/m/d) Food Tech Startup | 14-20h/Woche</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://planetafoods.jobs.personio.de/job/2755621</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Assistant to the executive Board (m/w/d)</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D3" t="n">
         <v>7</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Garching</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2706851</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Community Manager (m/w/d) - Front Desk MakerSpace Garching</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D4" t="n">
         <v>7</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Garching</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2709394</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr"/>
-      <c r="B4" s="3" t="inlineStr">
+    <row r="5">
+      <c r="B5" t="inlineStr">
         <is>
           <t>Robert Half Munich (All roles)</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Sachbearbeiter Export (w/m/d)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D5" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>...rbeiter Export (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-export-wmd/06640-0013462604-dede</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="inlineStr"/>
-      <c r="B5" s="3" t="inlineStr">
+    <row r="6">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Robert Half Munich (All roles)</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D6" t="n">
         <v>5</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013475955-dede</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Randstad Germany (Nachhaltigkeit)</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>Sachbearbeiter</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-sachbearbeiter/</t>
         </is>
       </c>
     </row>
@@ -876,25 +873,25 @@
       <c r="A7" s="3" t="inlineStr"/>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Randstad Germany (Nachhaltigkeit)</t>
+          <t>Robert Half Munich (Assistenz)</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Call Center Agent</t>
+          <t>Assistent Personalabteilung</t>
         </is>
       </c>
       <c r="D7" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+          <t>...fentlichen Dienst mit Sitz in München, zum nächstmöglichen Zeitpunk...</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>https://www.randstad.de/jobs/b-dienstleistung-und-service/j-call-center-agent/</t>
+          <t>https://www.roberthalf.com/de/de/job/deutschland/assistent-personalabteilung/06604-0013487193-dede</t>
         </is>
       </c>
     </row>
@@ -902,389 +899,375 @@
       <c r="A8" s="3" t="inlineStr"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>Tempton Personaldienstleistungen</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>12.08.2026 Personalsachbearbeiter / kaufmännischer Mitarbeiterin Lohn und Gehalt / Bürokauffrau (m/w/d) München</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>...n auf LinkedIn Jetzt bewerben München , Vollzeit Personalsachbearbe...</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tempton.de/karriere-intern/jobs/personalsachbearbeiter-kaufmaennischer-mitarbeiterin-lohn-gehalt-buerokauffrau</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-sachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Call Center Agent</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-dienstleistung-und-service/j-call-center-agent/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
         <is>
           <t>Sachbearbeiter Buchhaltung</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D11" t="n">
         <v>3</v>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-finanz-und-rechnungswesen/t-rechnungswesen/j-sachbearbeiter-buchhaltung/</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr"/>
-      <c r="B9" s="3" t="inlineStr">
+    <row r="12">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Auftragssachbearbeiter</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D12" t="n">
         <v>3</v>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-marketing-und-vertrieb/t-vertrieb-und-verkauf/j-auftragssachbearbeiter/</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr">
+    <row r="13">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Assistenz</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D13" t="n">
         <v>3</v>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz/</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="3" t="inlineStr"/>
-      <c r="B11" s="3" t="inlineStr">
+    <row r="14">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Assistenz der Geschäftsführung</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D14" t="n">
         <v>3</v>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz-der-geschaeftsfuehrung/</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr"/>
-      <c r="B12" s="3" t="inlineStr">
+    <row r="15">
+      <c r="B15" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Bürokaufmann</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D15" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-buerokaufmann/</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr"/>
-      <c r="B13" s="3" t="inlineStr">
+    <row r="16">
+      <c r="B16" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Empfangsmitarbeiter</t>
         </is>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D16" t="n">
         <v>3</v>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-empfangsmitarbeiter/</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr"/>
-      <c r="B14" s="3" t="inlineStr">
+    <row r="17">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Personalsachbearbeiter</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D17" t="n">
         <v>3</v>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-personalwesen/j-personalsachbearbeiter/</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
-      <c r="B15" s="3" t="inlineStr">
+    <row r="18">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Projektassistenz</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D18" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-projektassistenz/</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="3" t="inlineStr">
+    <row r="19">
+      <c r="B19" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Sachbearbeiter</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D19" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-sachbearbeiter/</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="3" t="inlineStr">
+    <row r="20">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Randstad Germany (Nachhaltigkeit)</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Verwaltungsfachangestellter</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D20" t="n">
         <v>3</v>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-verwaltungsfachangestellter/</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="3" t="inlineStr">
+    <row r="21">
+      <c r="B21" t="inlineStr">
         <is>
           <t>Robert Half Munich (All roles)</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D21" t="n">
         <v>3</v>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013471891-dede</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="3" t="inlineStr">
+    <row r="22">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Randstad Germany (Munich, all roles)</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Management-Assistenz (m/w/d)</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D22" t="n">
         <v>3</v>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>...nagement-Assistenz (m/w/d) in München | Randstad randstad Jobsuche...</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>https://www.randstad.de/jobs/management-assistenz-mwd_muenchen_c01310721/</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr"/>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>Michael Page Germany (Nachhaltigkeit)</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Facility Management</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
-        </is>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>https://www.michaelpage.de/jobs/facility-management</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Michael Page Germany (Nachhaltigkeit)</t>
-        </is>
-      </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>Sales Support &amp; Customer Service</t>
-        </is>
-      </c>
-      <c r="D21" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E21" s="3" t="inlineStr">
-        <is>
-          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
-        </is>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
-        <is>
-          <t>https://www.michaelpage.de/jobs/sales-support-customer-service</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Amadeus Fire (Munich)</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>Backoffice</t>
-        </is>
-      </c>
-      <c r="D22" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="E22" s="3" t="inlineStr">
-        <is>
-          <t>...e Köln Leipzig Mainz Mannheim München Münster Nürnberg Stuttgart Fa...</t>
-        </is>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>https://karriere.amadeus-fire.de/backoffice</t>
         </is>
       </c>
     </row>
@@ -1292,103 +1275,100 @@
       <c r="A23" s="3" t="inlineStr"/>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>Robert Half Munich (Assistenz)</t>
+          <t>Manpower Germany (Munich)</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>Assistenz des Gesamtbetriebsrats ( w/m/d)</t>
+          <t>Teamassistenz (m/w/d) Empfang &amp; Recht</t>
         </is>
       </c>
       <c r="D23" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>...tbetriebsrats ( w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+          <t>...nz (m/w/d) Empfang &amp; Recht in München | Manpower Germany (Deutsch)...</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
-          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/assistenz-des-gesamtbetriebsrats-wmd/06604-0013483434-dede</t>
+          <t>https://www.manpower.de/de/jobs/industry/teamassistenz-mwd-empfang-recht/35cf1dec-3f0c-4a32-a28e-dd12519a8612</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr"/>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>Robert Half Munich (Assistenz)</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>HR Assistent (w/m/d)</t>
-        </is>
-      </c>
-      <c r="D24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>HR Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
-        </is>
-      </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013482368-dede</t>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Facility Management</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/facility-management</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr"/>
-      <c r="B25" s="3" t="inlineStr">
-        <is>
-          <t>Robert Half Munich (Assistenz)</t>
-        </is>
-      </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>HR-Assistent (w/m/d)</t>
-        </is>
-      </c>
-      <c r="D25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E25" s="3" t="inlineStr">
-        <is>
-          <t>HR-Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
-        </is>
-      </c>
-      <c r="F25" s="3" t="inlineStr">
-        <is>
-          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013479384-dede</t>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Sales Support &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/sales-support-customer-service</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr"/>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>Robert Half Munich (Assistenz)</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>Sekretär der Führungsebene (w/m/d)</t>
-        </is>
-      </c>
-      <c r="D26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>...Führungsebene (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
-        </is>
-      </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sekretär-der-führungsebene-wmd/06604-0013471824-dede</t>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Amadeus Fire (Munich)</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Backoffice</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>2</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>...e Köln Leipzig Mainz Mannheim München Münster Nürnberg Stuttgart Fa...</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://karriere.amadeus-fire.de/backoffice</t>
         </is>
       </c>
     </row>
@@ -1396,25 +1376,25 @@
       <c r="A27" s="3" t="inlineStr"/>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Robert Half Munich (All roles)</t>
+          <t>Manpower Germany (Munich)</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>Kreditsachbearbeiter (w/m/d)</t>
+          <t>Sachbearbeiter Kredit- und Bürgschaftsmanagement (m/w/d)</t>
         </is>
       </c>
       <c r="D27" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E27" s="3" t="inlineStr">
         <is>
-          <t>...sachbearbeiter (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+          <t>...gschaftsmanagement (m/w/d) in München | Manpower Germany (Deutsch)...</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/kreditsachbearbeiter-wmd/06644-0013484134-dede</t>
+          <t>https://www.manpower.de/de/jobs/banken/sachbearbeiter-kredit-und-brgschaftsmanagement-mwd-/047b5a6f-dc78-459e-a025-62d811fa09f6</t>
         </is>
       </c>
     </row>
@@ -1422,23 +1402,173 @@
       <c r="A28" s="3" t="inlineStr"/>
       <c r="B28" s="3" t="inlineStr">
         <is>
+          <t>Manpower Germany (Munich)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Markensachbearbeiter / Trademark Paralegal (gn)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>...Trademark Paralegal (gn)  in München | Manpower Germany (Deutsch)...</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.manpower.de/de/jobs/industry/markensachbearbeiter-trademark-paralegal-gn-/69f6f741-003a-44e5-a5f5-56404a363040</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Assistenz des Gesamtbetriebsrats ( w/m/d)</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>...tbetriebsrats ( w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/assistenz-des-gesamtbetriebsrats-wmd/06604-0013483434-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013482368-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013479384-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Sekretär der Führungsebene (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>...Führungsebene (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sekretär-der-führungsebene-wmd/06604-0013471824-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" t="inlineStr">
+        <is>
           <t>Robert Half Munich (All roles)</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Kreditsachbearbeiter (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>...sachbearbeiter (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/kreditsachbearbeiter-wmd/06644-0013484134-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
         <is>
           <t>Technische Vertriebsassistenz (w/m/d)</t>
         </is>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D34" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>...riebsassistenz (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>https://www.roberthalf.com/de/de/job/münchen-bayern/technische-vertriebsassistenz-wmd/06604-0013485530-dede</t>
         </is>
@@ -1499,442 +1629,425 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr"/>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>5 C CarbonPlan 1 job 118</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" t="n">
         <v>4</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/carbonplan</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr"/>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>6 F FirstCarbon Solutions (FCS), an ADEC Innovation 1 job 113</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" t="n">
         <v>4</v>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/firstcarbon-solutions-fcs-an-adec-innovation</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr"/>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Climate Jobs</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://climate.jobs/</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr"/>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>Sustainability</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs?q=Sustainability</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>ESG &amp; Carbon</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs/category/esg-reporting-carbon</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Carbon</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs?q=Carbon</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Climate Policy</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" t="n">
         <v>2</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs/category/advocacy-policy</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>2 C Climate Collective Foundation 1 job 320</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" t="n">
         <v>2</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/climate-collective-foundation</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>3 C Climate Action Reserve 2 jobs 164</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" t="n">
         <v>2</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/climateactionreserve</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>4 G goodcarbon 3 jobs 127</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" t="n">
         <v>2</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/goodcarbon-earth</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>7 C ClimateWorks Foundation 2 jobs 109</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/climateworks</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>EuroClimateJobs.com</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Carbon Capture and Storage (15)</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>https://www.euroclimatejobs.com/jobs/carbon_capture_and_storage</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>EuroClimateJobs.com</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Climate and Energy Analyst (27)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>https://www.euroclimatejobs.com/jobs/climate_and_energy_analyst</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="4" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C15" s="4" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>Remote Climate Jobs</t>
         </is>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" t="n">
         <v>1</v>
       </c>
-      <c r="E15" s="4" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F15" s="4" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=inline&amp;utm_campaign=upgrade&amp;utm_content=homepage-how-it-works</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="4" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C16" s="4" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Remote Climate Jobs</t>
         </is>
       </c>
-      <c r="D16" s="4" t="n">
+      <c r="D16" t="n">
         <v>1</v>
       </c>
-      <c r="E16" s="4" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=faq&amp;utm_campaign=upgrade&amp;utm_content=homepage-faq-locked</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr"/>
-      <c r="B17" s="4" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C17" s="4" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Remote Climate Jobs Newsletter</t>
         </is>
       </c>
-      <c r="D17" s="4" t="n">
+      <c r="D17" t="n">
         <v>1</v>
       </c>
-      <c r="E17" s="4" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F17" s="4" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=footer&amp;utm_campaign=upgrade&amp;utm_content=footer</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="4" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C18" s="4" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Why climate.jobs?</t>
         </is>
       </c>
-      <c r="D18" s="4" t="n">
+      <c r="D18" t="n">
         <v>1</v>
       </c>
-      <c r="E18" s="4" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>https://climate.jobs/why-climate-jobs</t>
         </is>

</xml_diff>

<commit_message>
Update job tracker 2026-08-24 20:46 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +43,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
+        <bgColor rgb="00FDE68A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,9 +76,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -469,6 +490,140 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CSR Jobs in München</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>...punkt Immobilien (m|w|d) MEAG MUNICH ERGO AssetManagement GmbH | M...</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/csr-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Associate Sustainability Specialist (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2644410</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Nachhaltigkeit</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/nachhaltigkeit</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>BUND Naturschutz in Bayern</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Referent*in für Klimaschutz und Energie (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/referentin-fuer-klimaschutz-und-energie-m/w/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München | NachhaltigeJobs Nachhaltige...</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/umwelt-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -480,7 +635,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -523,6 +678,824 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Planet A Foods</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Office Management &amp; HR - Werkstudent (f/m/d) Food Tech Startup | 14-20h/Woche</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://planetafoods.jobs.personio.de/job/2755621</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Assistant to the executive Board (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Garching</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2706851</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Community Manager (m/w/d) - Front Desk MakerSpace Garching</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Garching</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2709394</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Assistent Personalabteilung</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>...fentlichen Dienst mit Sitz in München, zum nächstmöglichen Zeitpunk...</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/deutschland/assistent-personalabteilung/06604-0013487193-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Export (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>...rbeiter Export (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-export-wmd/06640-0013462604-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013475955-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tempton Personaldienstleistungen</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>12.08.2026 Personalsachbearbeiter / kaufmännischer Mitarbeiterin Lohn und Gehalt / Bürokauffrau (m/w/d) München</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>...n auf LinkedIn Jetzt bewerben München , Vollzeit Personalsachbearbe...</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tempton.de/karriere-intern/jobs/personalsachbearbeiter-kaufmaennischer-mitarbeiterin-lohn-gehalt-buerokauffrau</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-sachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Buchhaltung</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-finanz-und-rechnungswesen/t-rechnungswesen/j-sachbearbeiter-buchhaltung/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Auftragssachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-marketing-und-vertrieb/t-vertrieb-und-verkauf/j-auftragssachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz der Geschäftsführung</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz-der-geschaeftsfuehrung/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Bürokaufmann</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-buerokaufmann/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Empfangsmitarbeiter</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-empfangsmitarbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Personalsachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-personalwesen/j-personalsachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Projektassistenz</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-projektassistenz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-sachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Einkauf</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-sachbearbeiter-einkauf/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Verwaltungsfachangestellter</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-verwaltungsfachangestellter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013471891-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Munich, all roles)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Management-Assistenz (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>...nagement-Assistenz (m/w/d) in München | Randstad randstad Jobsuche...</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/management-assistenz-mwd_muenchen_c01310721/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Facility Management</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/facility-management</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Michael Page Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Sales Support &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>...üsseldorf Frankfurt Stuttgart München Alle Büros Kontakt Kontakt au...</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.michaelpage.de/jobs/sales-support-customer-service</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Amadeus Fire (Munich)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Backoffice</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>...e Köln Leipzig Mainz Mannheim München Münster Nürnberg Stuttgart Fa...</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>https://karriere.amadeus-fire.de/backoffice</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz des Gesamtbetriebsrats ( w/m/d)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>...tbetriebsrats ( w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/assistenz-des-gesamtbetriebsrats-wmd/06604-0013483434-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/assistent-wmd/06604-0013490419-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013482368-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013479384-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Sekretär der Führungsebene (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>...Führungsebene (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sekretär-der-führungsebene-wmd/06604-0013471824-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr"/>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
+          <t>Kreditsachbearbeiter (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>...sachbearbeiter (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/kreditsachbearbeiter-wmd/06644-0013484134-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Technische Vertriebsassistenz (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>...riebsassistenz (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/technische-vertriebsassistenz-wmd/06604-0013485530-dede</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -534,7 +1507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,6 +1550,370 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>6 C CarbonPlan 1 job 194</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/carbonplan</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>ESG &amp; Carbon</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/esg-reporting-carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Sustainability</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Sustainability</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1 C Climate Collective Foundation 1 job 515</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climate-collective-foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>8 C Climate Action Reserve 2 jobs 139</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climateactionreserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>9 C Climate Equity Fund (Equity Fund) 1 job 127</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/equityfund</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Carbon Capture and Storage (19)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/carbon_capture_and_storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Climate and Energy Analyst (23)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/climate_and_energy_analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Climate Policy</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/advocacy-policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=inline&amp;utm_campaign=upgrade&amp;utm_content=homepage-how-it-works</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=faq&amp;utm_campaign=upgrade&amp;utm_content=homepage-faq-locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs Newsletter</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=footer&amp;utm_campaign=upgrade&amp;utm_content=footer</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Why climate.jobs?</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/why-climate-jobs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-25 06:14 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +43,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
+        <bgColor rgb="00FDE68A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,9 +76,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -469,6 +490,114 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>CSR Jobs in München</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>...punkt Immobilien (m|w|d) MEAG MUNICH ERGO AssetManagement GmbH | M...</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/csr-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Associate Sustainability Specialist (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2644410</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>BUND Naturschutz in Bayern</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Referent*in für Klimaschutz und Energie (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/referentin-fuer-klimaschutz-und-energie-m/w/d</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>NachhaltigeJobs.de (Munich)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Umwelt Jobs in München | NachhaltigeJobs Nachhaltige...</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nachhaltigejobs.de/umwelt-jobs/muenchen</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -480,7 +609,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -523,6 +652,772 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Planet A Foods</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Office Management &amp; HR - Werkstudent (f/m/d) Food Tech Startup | 14-20h/Woche</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://planetafoods.jobs.personio.de/job/2755621</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Assistant to the executive Board (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Garching</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2706851</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Community Manager (m/w/d) - Front Desk MakerSpace Garching</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Garching</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2709394</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr"/>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Assistent Personalabteilung</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>...fentlichen Dienst mit Sitz in München, zum nächstmöglichen Zeitpunk...</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/deutschland/assistent-personalabteilung/06604-0013487193-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Export (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>...rbeiter Export (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-export-wmd/06640-0013462604-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013475955-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Tempton Personaldienstleistungen</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>12.08.2026 Personalsachbearbeiter / kaufmännischer Mitarbeiterin Lohn und Gehalt / Bürokauffrau (m/w/d) München</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>...n auf LinkedIn Jetzt bewerben München , Vollzeit Personalsachbearbe...</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://www.tempton.de/karriere-intern/jobs/personalsachbearbeiter-kaufmaennischer-mitarbeiterin-lohn-gehalt-buerokauffrau</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr"/>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-sachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Buchhaltung</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-finanz-und-rechnungswesen/t-rechnungswesen/j-sachbearbeiter-buchhaltung/</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr"/>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Auftragssachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-marketing-und-vertrieb/t-vertrieb-und-verkauf/j-auftragssachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr"/>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz der Geschäftsführung</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-assistenz-der-geschaeftsfuehrung/</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Bürokaufmann</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-buerokaufmann/</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr"/>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Empfangsmitarbeiter</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-empfangsmitarbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Personalsachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-personalwesen/j-personalsachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Projektassistenz</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-projektassistenz/</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-sachbearbeiter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Einkauf</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/t-administration-und-verwaltung/j-sachbearbeiter-einkauf/</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Nachhaltigkeit)</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Verwaltungsfachangestellter</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>...am Main Hamburg Köln Leipzig München Stuttgart Top Suchbegriffe La...</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/b-wirtschaft-und-administration/j-verwaltungsfachangestellter/</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Sachbearbeiter Kreditorenbuchhaltung (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>...renbuchhaltung (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sachbearbeiter-kreditorenbuchhaltung-wmd/06640-0013471891-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Randstad Germany (Munich, all roles)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Management-Assistenz (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>...nagement-Assistenz (m/w/d) in München | Randstad randstad Jobsuche...</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.randstad.de/jobs/management-assistenz-mwd_muenchen_c01310721/</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr"/>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Amadeus Fire (Munich)</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Backoffice</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>...e Köln Leipzig Mainz Mannheim München Münster Nürnberg Stuttgart Fa...</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>https://karriere.amadeus-fire.de/backoffice</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Assistenz des Gesamtbetriebsrats ( w/m/d)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>...tbetriebsrats ( w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/assistenz-des-gesamtbetriebsrats-wmd/06604-0013483434-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/assistent-wmd/06604-0013490419-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>HR Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013482368-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>HR-Assistent (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/hr-assistent-wmd/06640-0013479384-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (Assistenz)</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Sekretär der Führungsebene (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>...Führungsebene (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/sekretär-der-führungsebene-wmd/06604-0013471824-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>Kreditsachbearbeiter (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>...sachbearbeiter (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/kreditsachbearbeiter-wmd/06644-0013484134-dede</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Robert Half Munich (All roles)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Technische Vertriebsassistenz (w/m/d)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>...riebsassistenz (w/m/d) Job in München, Bayern | Robert Half Jobsuch...</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>https://www.roberthalf.com/de/de/job/münchen-bayern/technische-vertriebsassistenz-wmd/06604-0013485530-dede</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -534,7 +1429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,6 +1472,370 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>ESG &amp; Carbon</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/esg-reporting-carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>6 C CarbonPlan 1 job 199</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/carbonplan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Sustainability</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Sustainability</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>1 C Climate Collective Foundation 1 job 514</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climate-collective-foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>8 C Climate Action Reserve 2 jobs 140</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climateactionreserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>9 C Climate Equity Fund (Equity Fund) 1 job 130</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/equityfund</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Carbon Capture and Storage (19)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/carbon_capture_and_storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Climate and Energy Analyst (23)</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/climate_and_energy_analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Climate Policy</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/advocacy-policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=inline&amp;utm_campaign=upgrade&amp;utm_content=homepage-how-it-works</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=faq&amp;utm_campaign=upgrade&amp;utm_content=homepage-faq-locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs Newsletter</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=footer&amp;utm_campaign=upgrade&amp;utm_content=footer</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>Why climate.jobs?</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E15" s="4" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/why-climate-jobs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-27 17:42 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -32,7 +32,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -43,6 +43,24 @@
       <patternFill patternType="solid">
         <fgColor rgb="001F2937"/>
         <bgColor rgb="001F2937"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
+        <bgColor rgb="00D1FAE5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FDE68A"/>
+        <bgColor rgb="00FDE68A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DBEAFE"/>
+        <bgColor rgb="00DBEAFE"/>
       </patternFill>
     </fill>
   </fills>
@@ -58,9 +76,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -426,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -469,6 +490,62 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-21</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Associate Sustainability Specialist (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2644410</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>BUND Naturschutz in Bayern</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Referent*in für Klimaschutz und Energie (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/referentin-fuer-klimaschutz-und-energie-m/w/d</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -480,7 +557,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -523,6 +600,768 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Celonis</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Intern / Working Student Online Training Translation (Korean speaking)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Munich, Germany</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/celonis/jobs/7886106003?gh_jid=7886106003</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-11</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>UVC Partners: Junior Value Creation Analyst - Intern or Working Student (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>München Kreativquartier</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2750389</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Praktikant:in Accelerator Programme (RESPOND Energy &amp; Urban)</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>München Kreativquartier</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2709291</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>UVC Partners: Data &amp; AI - Master Thesis / Internship (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>München Kreativquartier</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2769065</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Tanso</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Sales Intern (f/m/x)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>https://tanso.jobs.personio.de/job/2636858</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr"/>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Siqens</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Bachelorand / Masterand / Praktikant (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>https://www.sfc.com/de/karriere/stellenanzeige/initiativbewerbung-bachelorand-masterand-praktikant-id94-104/</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Feldwerke</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Intern - Finance &amp; Controlling (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>München (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>https://feldwerke.jobs.personio.de/job/2748370</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>2024-01-19</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Unsolicited Application: Intern or Working Student for our Investment Team at UVC</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>München Kreativquartier</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/1395193</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>BUND Naturschutz in Bayern</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Praktikum beim BUND Naturschutz</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/praktikum</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>NuuEnergy</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Praktikant/Werkstudent (m/w/d) People &amp; Culture</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>München</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>https://nuuenergy.jobs.personio.de/job/2761280</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-26</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Feldwerke</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>(Intern) Business Development (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>München (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>https://feldwerke.jobs.personio.de/job/2440947</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-26</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Feldwerke</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>(Intern) Entrepreneur in Residence (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>München (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>https://feldwerke.jobs.personio.de/job/2440935</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2025-11-26</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Feldwerke</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>(Intern) Founders Associate (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>München (Hybrid)</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>https://feldwerke.jobs.personio.de/job/2440850</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>2025-12-19</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>UnternehmerTUM Company Partners: Praktikant_in (m/w/d) für Innovationsprojekte</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>München Kreativquartier</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>https://unternehmertum.jobs.personio.de/job/2468855</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>HAWE Hydraulik SE</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Schülerpraktikum</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>...&amp; Benefits Standorte Aschheim-München Barbing Freising Kaufbeuren S...</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>https://hawe.com/de-de/unternehmen/karriere/ausbildung/schuelerpraktikum/</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr"/>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>BayernLB</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Traineeprogramm Vielfältige Einsatzbereiche, individuelle Entwicklung. Wir haben das passende Traineeprogramm für Dich!</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>...e moderne Kantine am Standort München Sportclub am Englischen Garte...</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bayernlb.de/internet/de/blb/resp/karriere_1/studenten_und_berufseinsteiger/traineeprogramm/trainees_2024.jsp</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>The Mobility House</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Werkstudent (m/w/d) Kreditorenbuchhaltung Praktikum/Werkstudium München</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>...eilzeit Praktikum/Werkstudium München Warum The Mobility House? Mit...</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2701912/werkstudent-mwd-kreditorenbuchhaltung</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr"/>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>The Mobility House</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>Werkstudent:in Projektmanagement Ladeinfrastruktur (m/w/d) Praktikum/Werkstudium München</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>...eilzeit Praktikum/Werkstudium München Warum The Mobility House? Mit...</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2717018/werkstudentin-projektmanagement-ladeinfrastruktur-mwd</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2024-12-18</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Planet A Foods</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Marketing Praktikant:in (f/m/d)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://planetafoods.jobs.personio.de/job/1881523</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>BayernLB</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>Praktikum und Abschlussarbeit</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>...finden in unserer Zentrale in München statt. Du kannst dich drei bi...</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>https://www.bayernlb.de/internet/de/blb/resp/karriere_1/studenten_und_berufseinsteiger/praktikum_und_abschlussarbeit_3/praktikum_und_werkstudenten.jsp</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Stadtwerke Muenchen</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Ausbildung | Schülerpraktikum</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>...hstarten? Bei den Stadtwerken München (SWM) arbeitest du nicht nur...</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>https://www.swm.de/karriere/berufseinsteiger/ausbildung</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>2024-08-27</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>FINN</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Internship - B2B Sales (m/w/d)</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>https://jobs.lever.co/finn/fc5d1573-a0ef-4152-804f-099fb622b3b8</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>2024-06-03</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>AMSilk</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Internship or Master’s Thesis in Downstream Process Development (6 months)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Neuried</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>https://amsilk.jobs.personio.de/job/1585005</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr"/>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Amadeus Fire (Munich)</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>Praktikum</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>...e Köln Leipzig Mainz Mannheim München Münster Nürnberg Stuttgart Fa...</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>https://karriere.amadeus-fire.de/praktikum</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>I.K. Hofmann / experts (Munich)</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Interne Stellenangebote</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>...r Magdeburg Frankfurt Leipzig München Nürnberg Regensburg Zwickau F...</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>https://experts.jobs/bewerber/interne-stellenangebote/</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr"/>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Bavarian International School (BIS)</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Open Positions at BAVARIAN INTERNATIONAL SCHOOL</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Munich</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>https://bis.jobs.personio.de/</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>AeroGround Flughafen München GmbH</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Initiativbewerbung für ein Hochschulpraktikum</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>...nschutz Newsletter ©Flughafen München GmbH powered by d.vinci</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>https://bewerben.munich-airport.de/de/jobs/382/intro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -534,7 +1373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -577,6 +1416,344 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" s="4" t="inlineStr"/>
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C2" s="4" t="inlineStr">
+        <is>
+          <t>Sustainability</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>...k all → Search All work types Remote (1) On-site (29) Hybrid (46)...</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Sustainability</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr"/>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>ESG &amp; Carbon</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>...k all → Search All work types Remote (3) On-site (53) Hybrid (68)...</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/esg-reporting-carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr"/>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Carbon</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>...k all → Search All work types Remote (5) On-site (71) Hybrid (82)...</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs?q=Carbon</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr"/>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2 C Climate Collective Foundation 1 job 489</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>...ganizational objectives. Work remotely (location not specified) Re...</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climate-collective-foundation</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr"/>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>7 C Climate Action Reserve 2 jobs 146</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>...travel to project sites. Work remotely from United States Remote 🌍...</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/climateactionreserve</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr"/>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>8 C Climate Equity Fund (Equity Fund) 1 job 142</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>...nd fundraising outreach. Work remotely from United States Remote 📣...</t>
+        </is>
+      </c>
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/company/equityfund</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>Carbon Capture and Storage (19)</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>...lace Hybrid (54) On-site (82) Remote (7) Jobs By Location Austria...</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/carbon_capture_and_storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr"/>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>EuroClimateJobs.com</t>
+        </is>
+      </c>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>Climate and Energy Analyst (24)</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>...lace Hybrid (54) On-site (82) Remote (7) Jobs By Location Austria...</t>
+        </is>
+      </c>
+      <c r="F9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.euroclimatejobs.com/jobs/climate_and_energy_analyst</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr"/>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>Climate Policy</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>...k all → Search All work types Remote (11) On-site (6) Hybrid (9) A...</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/jobs/category/advocacy-policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>Home | Remote Climate Jobs Remote Climate J...</t>
+        </is>
+      </c>
+      <c r="F11" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=inline&amp;utm_campaign=upgrade&amp;utm_content=homepage-how-it-works</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="4" t="inlineStr"/>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Home | Remote Climate Jobs Remote Climate J...</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=faq&amp;utm_campaign=upgrade&amp;utm_content=homepage-faq-locked</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Remote Climate Jobs Newsletter</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>Home | Remote Climate Jobs Remote Climate J...</t>
+        </is>
+      </c>
+      <c r="F13" s="4" t="inlineStr">
+        <is>
+          <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=footer&amp;utm_campaign=upgrade&amp;utm_content=footer</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>climate.jobs (remote)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Why climate.jobs?</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>...limate since 2023 through the Remote Climate Jobs newsletter - whi...</t>
+        </is>
+      </c>
+      <c r="F14" s="4" t="inlineStr">
+        <is>
+          <t>https://climate.jobs/why-climate-jobs</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update job tracker 2026-08-27 18:39 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -491,56 +491,55 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-05-21</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Tanso</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Associate Sustainability Specialist (f/m/x)</t>
         </is>
       </c>
-      <c r="D2" s="2" t="n">
+      <c r="D2" t="n">
         <v>6</v>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://tanso.jobs.personio.de/job/2644410</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr"/>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>BUND Naturschutz in Bayern</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>Referent*in für Klimaschutz und Energie (m/w/d)</t>
         </is>
       </c>
-      <c r="D3" s="2" t="n">
+      <c r="D3" t="n">
         <v>1</v>
       </c>
-      <c r="E3" s="2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F3" s="2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/referentin-fuer-klimaschutz-und-energie-m/w/d</t>
         </is>
@@ -601,762 +600,750 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="3" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>2026-08-25</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>Celonis</t>
         </is>
       </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Intern / Working Student Online Training Translation (Korean speaking)</t>
         </is>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" t="n">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>Munich, Germany</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://job-boards.greenhouse.io/celonis/jobs/7886106003?gh_jid=7886106003</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" t="inlineStr">
         <is>
           <t>2026-08-11</t>
         </is>
       </c>
-      <c r="B3" s="3" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>UVC Partners: Junior Value Creation Analyst - Intern or Working Student (f/m/x)</t>
         </is>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" t="n">
         <v>8</v>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>München Kreativquartier</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2750389</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" t="inlineStr">
         <is>
           <t>2026-07-13</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Praktikant:in Accelerator Programme (RESPOND Energy &amp; Urban)</t>
         </is>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" t="n">
         <v>7</v>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>München Kreativquartier</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2709291</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
+      <c r="A5" t="inlineStr">
         <is>
           <t>2026-08-26</t>
         </is>
       </c>
-      <c r="B5" s="3" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C5" s="3" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>UVC Partners: Data &amp; AI - Master Thesis / Internship (f/m/x)</t>
         </is>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" t="n">
         <v>7</v>
       </c>
-      <c r="E5" s="3" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>München Kreativquartier</t>
         </is>
       </c>
-      <c r="F5" s="3" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2769065</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" t="inlineStr">
         <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>Tanso</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>Sales Intern (f/m/x)</t>
         </is>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://tanso.jobs.personio.de/job/2636858</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr"/>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Siqens</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Bachelorand / Masterand / Praktikant (m/w/d)</t>
         </is>
       </c>
-      <c r="D7" s="3" t="n">
+      <c r="D7" t="n">
         <v>7</v>
       </c>
-      <c r="E7" s="3" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://www.sfc.com/de/karriere/stellenanzeige/initiativbewerbung-bachelorand-masterand-praktikant-id94-104/</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" t="inlineStr">
         <is>
           <t>2026-08-10</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>Feldwerke</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Intern - Finance &amp; Controlling (m/w/d)</t>
         </is>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D8" t="n">
         <v>6</v>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>München (Hybrid)</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://feldwerke.jobs.personio.de/job/2748370</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" t="inlineStr">
         <is>
           <t>2024-01-19</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Unsolicited Application: Intern or Working Student for our Investment Team at UVC</t>
         </is>
       </c>
-      <c r="D9" s="3" t="n">
+      <c r="D9" t="n">
         <v>5</v>
       </c>
-      <c r="E9" s="3" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>München Kreativquartier</t>
         </is>
       </c>
-      <c r="F9" s="3" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/1395193</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr"/>
-      <c r="B10" s="3" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>BUND Naturschutz in Bayern</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Praktikum beim BUND Naturschutz</t>
         </is>
       </c>
-      <c r="D10" s="3" t="n">
+      <c r="D10" t="n">
         <v>5</v>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/praktikum</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="3" t="inlineStr">
+      <c r="A11" t="inlineStr">
         <is>
           <t>2026-08-20</t>
         </is>
       </c>
-      <c r="B11" s="3" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>NuuEnergy</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Praktikant/Werkstudent (m/w/d) People &amp; Culture</t>
         </is>
       </c>
-      <c r="D11" s="3" t="n">
+      <c r="D11" t="n">
         <v>4</v>
       </c>
-      <c r="E11" s="3" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>München</t>
         </is>
       </c>
-      <c r="F11" s="3" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>https://nuuenergy.jobs.personio.de/job/2761280</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" t="inlineStr">
         <is>
           <t>2025-11-26</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>Feldwerke</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>(Intern) Business Development (m/w/d)</t>
         </is>
       </c>
-      <c r="D12" s="3" t="n">
+      <c r="D12" t="n">
         <v>4</v>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>München (Hybrid)</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>https://feldwerke.jobs.personio.de/job/2440947</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+      <c r="A13" t="inlineStr">
         <is>
           <t>2025-11-26</t>
         </is>
       </c>
-      <c r="B13" s="3" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>Feldwerke</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>(Intern) Entrepreneur in Residence (m/w/d)</t>
         </is>
       </c>
-      <c r="D13" s="3" t="n">
+      <c r="D13" t="n">
         <v>4</v>
       </c>
-      <c r="E13" s="3" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>München (Hybrid)</t>
         </is>
       </c>
-      <c r="F13" s="3" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>https://feldwerke.jobs.personio.de/job/2440935</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+      <c r="A14" t="inlineStr">
         <is>
           <t>2025-11-26</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Feldwerke</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>(Intern) Founders Associate (m/w/d)</t>
         </is>
       </c>
-      <c r="D14" s="3" t="n">
+      <c r="D14" t="n">
         <v>4</v>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>München (Hybrid)</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>https://feldwerke.jobs.personio.de/job/2440850</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+      <c r="A15" t="inlineStr">
         <is>
           <t>2025-12-19</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B15" t="inlineStr">
         <is>
           <t>UnternehmerTUM</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>UnternehmerTUM Company Partners: Praktikant_in (m/w/d) für Innovationsprojekte</t>
         </is>
       </c>
-      <c r="D15" s="3" t="n">
+      <c r="D15" t="n">
         <v>3</v>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E15" t="inlineStr">
         <is>
           <t>München Kreativquartier</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>https://unternehmertum.jobs.personio.de/job/2468855</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="3" t="inlineStr"/>
-      <c r="B16" s="3" t="inlineStr">
+      <c r="B16" t="inlineStr">
         <is>
           <t>HAWE Hydraulik SE</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>Schülerpraktikum</t>
         </is>
       </c>
-      <c r="D16" s="3" t="n">
+      <c r="D16" t="n">
         <v>3</v>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" t="inlineStr">
         <is>
           <t>...&amp; Benefits Standorte Aschheim-München Barbing Freising Kaufbeuren S...</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>https://hawe.com/de-de/unternehmen/karriere/ausbildung/schuelerpraktikum/</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
-      <c r="B17" s="3" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>BayernLB</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>Traineeprogramm Vielfältige Einsatzbereiche, individuelle Entwicklung. Wir haben das passende Traineeprogramm für Dich!</t>
         </is>
       </c>
-      <c r="D17" s="3" t="n">
+      <c r="D17" t="n">
         <v>2</v>
       </c>
-      <c r="E17" s="3" t="inlineStr">
+      <c r="E17" t="inlineStr">
         <is>
           <t>...e moderne Kantine am Standort München Sportclub am Englischen Garte...</t>
         </is>
       </c>
-      <c r="F17" s="3" t="inlineStr">
+      <c r="F17" t="inlineStr">
         <is>
           <t>https://www.bayernlb.de/internet/de/blb/resp/karriere_1/studenten_und_berufseinsteiger/traineeprogramm/trainees_2024.jsp</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="3" t="inlineStr"/>
-      <c r="B18" s="3" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>The Mobility House</t>
         </is>
       </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Werkstudent (m/w/d) Kreditorenbuchhaltung Praktikum/Werkstudium München</t>
         </is>
       </c>
-      <c r="D18" s="3" t="n">
+      <c r="D18" t="n">
         <v>2</v>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" t="inlineStr">
         <is>
           <t>...eilzeit Praktikum/Werkstudium München Warum The Mobility House? Mit...</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
+      <c r="F18" t="inlineStr">
         <is>
           <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2701912/werkstudent-mwd-kreditorenbuchhaltung</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr"/>
-      <c r="B19" s="3" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t>The Mobility House</t>
         </is>
       </c>
-      <c r="C19" s="3" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>Werkstudent:in Projektmanagement Ladeinfrastruktur (m/w/d) Praktikum/Werkstudium München</t>
         </is>
       </c>
-      <c r="D19" s="3" t="n">
+      <c r="D19" t="n">
         <v>2</v>
       </c>
-      <c r="E19" s="3" t="inlineStr">
+      <c r="E19" t="inlineStr">
         <is>
           <t>...eilzeit Praktikum/Werkstudium München Warum The Mobility House? Mit...</t>
         </is>
       </c>
-      <c r="F19" s="3" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2717018/werkstudentin-projektmanagement-ladeinfrastruktur-mwd</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" t="inlineStr">
         <is>
           <t>2024-12-18</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B20" t="inlineStr">
         <is>
           <t>Planet A Foods</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>Marketing Praktikant:in (f/m/d)</t>
         </is>
       </c>
-      <c r="D20" s="3" t="n">
+      <c r="D20" t="n">
         <v>2</v>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F20" t="inlineStr">
         <is>
           <t>https://planetafoods.jobs.personio.de/job/1881523</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
-      <c r="B21" s="3" t="inlineStr">
+      <c r="B21" t="inlineStr">
         <is>
           <t>BayernLB</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>Praktikum und Abschlussarbeit</t>
         </is>
       </c>
-      <c r="D21" s="3" t="n">
+      <c r="D21" t="n">
         <v>1</v>
       </c>
-      <c r="E21" s="3" t="inlineStr">
+      <c r="E21" t="inlineStr">
         <is>
           <t>...finden in unserer Zentrale in München statt. Du kannst dich drei bi...</t>
         </is>
       </c>
-      <c r="F21" s="3" t="inlineStr">
+      <c r="F21" t="inlineStr">
         <is>
           <t>https://www.bayernlb.de/internet/de/blb/resp/karriere_1/studenten_und_berufseinsteiger/praktikum_und_abschlussarbeit_3/praktikum_und_werkstudenten.jsp</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr"/>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B22" t="inlineStr">
         <is>
           <t>Stadtwerke Muenchen</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>Ausbildung | Schülerpraktikum</t>
         </is>
       </c>
-      <c r="D22" s="3" t="n">
+      <c r="D22" t="n">
         <v>1</v>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" t="inlineStr">
         <is>
           <t>...hstarten? Bei den Stadtwerken München (SWM) arbeitest du nicht nur...</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F22" t="inlineStr">
         <is>
           <t>https://www.swm.de/karriere/berufseinsteiger/ausbildung</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="3" t="inlineStr">
+      <c r="A23" t="inlineStr">
         <is>
           <t>2024-08-27</t>
         </is>
       </c>
-      <c r="B23" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>FINN</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>Internship - B2B Sales (m/w/d)</t>
         </is>
       </c>
-      <c r="D23" s="3" t="n">
+      <c r="D23" t="n">
         <v>1</v>
       </c>
-      <c r="E23" s="3" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F23" s="3" t="inlineStr">
+      <c r="F23" t="inlineStr">
         <is>
           <t>https://jobs.lever.co/finn/fc5d1573-a0ef-4152-804f-099fb622b3b8</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" t="inlineStr">
         <is>
           <t>2024-06-03</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>AMSilk</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>Internship or Master’s Thesis in Downstream Process Development (6 months)</t>
         </is>
       </c>
-      <c r="D24" s="3" t="n">
+      <c r="D24" t="n">
         <v>1</v>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" t="inlineStr">
         <is>
           <t>Neuried</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
+      <c r="F24" t="inlineStr">
         <is>
           <t>https://amsilk.jobs.personio.de/job/1585005</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="3" t="inlineStr"/>
-      <c r="B25" s="3" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>Amadeus Fire (Munich)</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>Praktikum</t>
         </is>
       </c>
-      <c r="D25" s="3" t="n">
+      <c r="D25" t="n">
         <v>1</v>
       </c>
-      <c r="E25" s="3" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>...e Köln Leipzig Mainz Mannheim München Münster Nürnberg Stuttgart Fa...</t>
         </is>
       </c>
-      <c r="F25" s="3" t="inlineStr">
+      <c r="F25" t="inlineStr">
         <is>
           <t>https://karriere.amadeus-fire.de/praktikum</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="3" t="inlineStr"/>
-      <c r="B26" s="3" t="inlineStr">
+      <c r="B26" t="inlineStr">
         <is>
           <t>I.K. Hofmann / experts (Munich)</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>Interne Stellenangebote</t>
         </is>
       </c>
-      <c r="D26" s="3" t="n">
+      <c r="D26" t="n">
         <v>1</v>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" t="inlineStr">
         <is>
           <t>...r Magdeburg Frankfurt Leipzig München Nürnberg Regensburg Zwickau F...</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
+      <c r="F26" t="inlineStr">
         <is>
           <t>https://experts.jobs/bewerber/interne-stellenangebote/</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="3" t="inlineStr"/>
-      <c r="B27" s="3" t="inlineStr">
+      <c r="B27" t="inlineStr">
         <is>
           <t>Bavarian International School (BIS)</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
+      <c r="C27" t="inlineStr">
         <is>
           <t>Open Positions at BAVARIAN INTERNATIONAL SCHOOL</t>
         </is>
       </c>
-      <c r="D27" s="3" t="n">
+      <c r="D27" t="n">
         <v>1</v>
       </c>
-      <c r="E27" s="3" t="inlineStr">
+      <c r="E27" t="inlineStr">
         <is>
           <t>Munich</t>
         </is>
       </c>
-      <c r="F27" s="3" t="inlineStr">
+      <c r="F27" t="inlineStr">
         <is>
           <t>https://bis.jobs.personio.de/</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="3" t="inlineStr"/>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>AeroGround Flughafen München GmbH</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Initiativbewerbung für ein Hochschulpraktikum</t>
         </is>
       </c>
-      <c r="D28" s="3" t="n">
+      <c r="D28" t="n">
         <v>1</v>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>...nschutz Newsletter ©Flughafen München GmbH powered by d.vinci</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>https://bewerben.munich-airport.de/de/jobs/382/intro</t>
         </is>
@@ -1417,338 +1404,325 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="4" t="inlineStr"/>
-      <c r="B2" s="4" t="inlineStr">
+      <c r="B2" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>Sustainability</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" t="n">
         <v>2</v>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" t="inlineStr">
         <is>
           <t>...k all → Search All work types Remote (1) On-site (29) Hybrid (46)...</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs?q=Sustainability</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr"/>
-      <c r="B3" s="4" t="inlineStr">
+      <c r="B3" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>ESG &amp; Carbon</t>
         </is>
       </c>
-      <c r="D3" s="4" t="n">
+      <c r="D3" t="n">
         <v>2</v>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>...k all → Search All work types Remote (3) On-site (53) Hybrid (68)...</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs/category/esg-reporting-carbon</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr"/>
-      <c r="B4" s="4" t="inlineStr">
+      <c r="B4" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>Carbon</t>
         </is>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" t="n">
         <v>2</v>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>...k all → Search All work types Remote (5) On-site (71) Hybrid (82)...</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs?q=Carbon</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr"/>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>2 C Climate Collective Foundation 1 job 489</t>
         </is>
       </c>
-      <c r="D5" s="4" t="n">
+      <c r="D5" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>...ganizational objectives. Work remotely (location not specified) Re...</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/climate-collective-foundation</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="4" t="inlineStr"/>
-      <c r="B6" s="4" t="inlineStr">
+      <c r="B6" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>7 C Climate Action Reserve 2 jobs 146</t>
         </is>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" t="n">
         <v>2</v>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>...travel to project sites. Work remotely from United States Remote 🌍...</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/climateactionreserve</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr"/>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>8 C Climate Equity Fund (Equity Fund) 1 job 142</t>
         </is>
       </c>
-      <c r="D7" s="4" t="n">
+      <c r="D7" t="n">
         <v>2</v>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>...nd fundraising outreach. Work remotely from United States Remote 📣...</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>https://climate.jobs/company/equityfund</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr"/>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" t="inlineStr">
         <is>
           <t>EuroClimateJobs.com</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>Carbon Capture and Storage (19)</t>
         </is>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" t="n">
         <v>1</v>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>...lace Hybrid (54) On-site (82) Remote (7) Jobs By Location Austria...</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>https://www.euroclimatejobs.com/jobs/carbon_capture_and_storage</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr"/>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>EuroClimateJobs.com</t>
         </is>
       </c>
-      <c r="C9" s="4" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>Climate and Energy Analyst (24)</t>
         </is>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" t="n">
         <v>1</v>
       </c>
-      <c r="E9" s="4" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>...lace Hybrid (54) On-site (82) Remote (7) Jobs By Location Austria...</t>
         </is>
       </c>
-      <c r="F9" s="4" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>https://www.euroclimatejobs.com/jobs/climate_and_energy_analyst</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C10" s="4" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>Climate Policy</t>
         </is>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" t="n">
         <v>1</v>
       </c>
-      <c r="E10" s="4" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>...k all → Search All work types Remote (11) On-site (6) Hybrid (9) A...</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>https://climate.jobs/jobs/category/advocacy-policy</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr"/>
-      <c r="B11" s="4" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C11" s="4" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>Remote Climate Jobs</t>
         </is>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" t="n">
         <v>1</v>
       </c>
-      <c r="E11" s="4" t="inlineStr">
+      <c r="E11" t="inlineStr">
         <is>
           <t>Home | Remote Climate Jobs Remote Climate J...</t>
         </is>
       </c>
-      <c r="F11" s="4" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=inline&amp;utm_campaign=upgrade&amp;utm_content=homepage-how-it-works</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="4" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C12" s="4" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>Remote Climate Jobs</t>
         </is>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" t="n">
         <v>1</v>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E12" t="inlineStr">
         <is>
           <t>Home | Remote Climate Jobs Remote Climate J...</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="F12" t="inlineStr">
         <is>
           <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=faq&amp;utm_campaign=upgrade&amp;utm_content=homepage-faq-locked</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="4" t="inlineStr">
+      <c r="B13" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C13" s="4" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>Remote Climate Jobs Newsletter</t>
         </is>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" t="n">
         <v>1</v>
       </c>
-      <c r="E13" s="4" t="inlineStr">
+      <c r="E13" t="inlineStr">
         <is>
           <t>Home | Remote Climate Jobs Remote Climate J...</t>
         </is>
       </c>
-      <c r="F13" s="4" t="inlineStr">
+      <c r="F13" t="inlineStr">
         <is>
           <t>https://remoteclimatejobs.co?utm_source=climate.jobs&amp;utm_medium=footer&amp;utm_campaign=upgrade&amp;utm_content=footer</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr"/>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>climate.jobs (remote)</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>Why climate.jobs?</t>
         </is>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" t="n">
         <v>1</v>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E14" t="inlineStr">
         <is>
           <t>...limate since 2023 through the Remote Climate Jobs newsletter - whi...</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="F14" t="inlineStr">
         <is>
           <t>https://climate.jobs/why-climate-jobs</t>
         </is>

</xml_diff>

<commit_message>
Update job tracker 2026-08-27 20:13 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -556,7 +556,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1346,6 +1346,32 @@
       <c r="F28" t="inlineStr">
         <is>
           <t>https://bewerben.munich-airport.de/de/jobs/382/intro</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr"/>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Munich Re</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>2026 Fall Intern</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>...dern Insurance Group, Inc., a Munich Re company, is a widely recog...</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.munichre.com/en/job/amelia/2026-fall-intern/3342/43229230208</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update job tracker 2026-08-27 21:02 UTC
</commit_message>
<xml_diff>
--- a/data/job_tracker.xlsx
+++ b/data/job_tracker.xlsx
@@ -602,17 +602,17 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Celonis</t>
+          <t>UnternehmerTUM</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Intern / Working Student Online Training Translation (Korean speaking)</t>
+          <t>UVC Partners: Junior Value Creation Analyst - Intern or Working Student (f/m/x)</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -620,19 +620,19 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Munich, Germany</t>
+          <t>München Kreativquartier</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://job-boards.greenhouse.io/celonis/jobs/7886106003?gh_jid=7886106003</t>
+          <t>https://unternehmertum.jobs.personio.de/job/2750389</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -642,11 +642,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>UVC Partners: Junior Value Creation Analyst - Intern or Working Student (f/m/x)</t>
+          <t>Praktikant:in Accelerator Programme (RESPOND Energy &amp; Urban)</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -655,14 +655,14 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://unternehmertum.jobs.personio.de/job/2750389</t>
+          <t>https://unternehmertum.jobs.personio.de/job/2709291</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -672,7 +672,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Praktikant:in Accelerator Programme (RESPOND Energy &amp; Urban)</t>
+          <t>UVC Partners: Data &amp; AI - Master Thesis / Internship (f/m/x)</t>
         </is>
       </c>
       <c r="D4" t="n">
@@ -685,24 +685,24 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://unternehmertum.jobs.personio.de/job/2709291</t>
+          <t>https://unternehmertum.jobs.personio.de/job/2769065</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>UnternehmerTUM</t>
+          <t>Tanso</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>UVC Partners: Data &amp; AI - Master Thesis / Internship (f/m/x)</t>
+          <t>Sales Intern (f/m/x)</t>
         </is>
       </c>
       <c r="D5" t="n">
@@ -710,29 +710,24 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>München Kreativquartier</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://unternehmertum.jobs.personio.de/job/2769065</t>
+          <t>https://tanso.jobs.personio.de/job/2636858</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tanso</t>
+          <t>Siqens</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Sales Intern (f/m/x)</t>
+          <t>Bachelorand / Masterand / Praktikant (m/w/d)</t>
         </is>
       </c>
       <c r="D6" t="n">
@@ -745,79 +740,79 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://tanso.jobs.personio.de/job/2636858</t>
+          <t>https://www.sfc.com/de/karriere/stellenanzeige/initiativbewerbung-bachelorand-masterand-praktikant-id94-104/</t>
         </is>
       </c>
     </row>
     <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-08-10</t>
+        </is>
+      </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Siqens</t>
+          <t>Feldwerke</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bachelorand / Masterand / Praktikant (m/w/d)</t>
+          <t>Intern - Finance &amp; Controlling (m/w/d)</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>München (Hybrid)</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://www.sfc.com/de/karriere/stellenanzeige/initiativbewerbung-bachelorand-masterand-praktikant-id94-104/</t>
+          <t>https://feldwerke.jobs.personio.de/job/2748370</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2024-01-19</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Feldwerke</t>
+          <t>UnternehmerTUM</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Intern - Finance &amp; Controlling (m/w/d)</t>
+          <t>Unsolicited Application: Intern or Working Student for our Investment Team at UVC</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>München (Hybrid)</t>
+          <t>München Kreativquartier</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://feldwerke.jobs.personio.de/job/2748370</t>
+          <t>https://unternehmertum.jobs.personio.de/job/1395193</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>2024-01-19</t>
-        </is>
-      </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>UnternehmerTUM</t>
+          <t>BUND Naturschutz in Bayern</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Unsolicited Application: Intern or Working Student for our Investment Team at UVC</t>
+          <t>Praktikum beim BUND Naturschutz</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -825,54 +820,59 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>München Kreativquartier</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://unternehmertum.jobs.personio.de/job/1395193</t>
+          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/praktikum</t>
         </is>
       </c>
     </row>
     <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-08-20</t>
+        </is>
+      </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>BUND Naturschutz in Bayern</t>
+          <t>NuuEnergy</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Praktikum beim BUND Naturschutz</t>
+          <t>Praktikant/Werkstudent (m/w/d) People &amp; Culture</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Munich</t>
+          <t>München</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://www.bund-naturschutz.de/ueber-uns/stellenangebote/praktikum</t>
+          <t>https://nuuenergy.jobs.personio.de/job/2761280</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2025-11-26</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>NuuEnergy</t>
+          <t>Feldwerke</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Praktikant/Werkstudent (m/w/d) People &amp; Culture</t>
+          <t>(Intern) Business Development (m/w/d)</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -880,12 +880,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>München</t>
+          <t>München (Hybrid)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://nuuenergy.jobs.personio.de/job/2761280</t>
+          <t>https://feldwerke.jobs.personio.de/job/2440947</t>
         </is>
       </c>
     </row>
@@ -902,7 +902,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>(Intern) Business Development (m/w/d)</t>
+          <t>(Intern) Entrepreneur in Residence (m/w/d)</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -915,7 +915,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://feldwerke.jobs.personio.de/job/2440947</t>
+          <t>https://feldwerke.jobs.personio.de/job/2440935</t>
         </is>
       </c>
     </row>
@@ -932,7 +932,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>(Intern) Entrepreneur in Residence (m/w/d)</t>
+          <t>(Intern) Founders Associate (m/w/d)</t>
         </is>
       </c>
       <c r="D13" t="n">
@@ -945,54 +945,49 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://feldwerke.jobs.personio.de/job/2440935</t>
+          <t>https://feldwerke.jobs.personio.de/job/2440850</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2025-11-26</t>
+          <t>2025-12-19</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Feldwerke</t>
+          <t>UnternehmerTUM</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>(Intern) Founders Associate (m/w/d)</t>
+          <t>UnternehmerTUM Company Partners: Praktikant_in (m/w/d) für Innovationsprojekte</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>München (Hybrid)</t>
+          <t>München Kreativquartier</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://feldwerke.jobs.personio.de/job/2440850</t>
+          <t>https://unternehmertum.jobs.personio.de/job/2468855</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>2025-12-19</t>
-        </is>
-      </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>UnternehmerTUM</t>
+          <t>HAWE Hydraulik SE</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>UnternehmerTUM Company Partners: Praktikant_in (m/w/d) für Innovationsprojekte</t>
+          <t>Schülerpraktikum</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -1000,49 +995,49 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>München Kreativquartier</t>
+          <t>...&amp; Benefits Standorte Aschheim-München Barbing Freising Kaufbeuren S...</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://unternehmertum.jobs.personio.de/job/2468855</t>
+          <t>https://hawe.com/de-de/unternehmen/karriere/ausbildung/schuelerpraktikum/</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>HAWE Hydraulik SE</t>
+          <t>BayernLB</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Schülerpraktikum</t>
+          <t>Traineeprogramm Vielfältige Einsatzbereiche, individuelle Entwicklung. Wir haben das passende Traineeprogramm für Dich!</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>...&amp; Benefits Standorte Aschheim-München Barbing Freising Kaufbeuren S...</t>
+          <t>...e moderne Kantine am Standort München Sportclub am Englischen Garte...</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://hawe.com/de-de/unternehmen/karriere/ausbildung/schuelerpraktikum/</t>
+          <t>https://www.bayernlb.de/internet/de/blb/resp/karriere_1/studenten_und_berufseinsteiger/traineeprogramm/trainees_2024.jsp</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" t="inlineStr">
         <is>
-          <t>BayernLB</t>
+          <t>The Mobility House</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Traineeprogramm Vielfältige Einsatzbereiche, individuelle Entwicklung. Wir haben das passende Traineeprogramm für Dich!</t>
+          <t>Werkstudent (m/w/d) Kreditorenbuchhaltung Praktikum/Werkstudium München</t>
         </is>
       </c>
       <c r="D17" t="n">
@@ -1050,12 +1045,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>...e moderne Kantine am Standort München Sportclub am Englischen Garte...</t>
+          <t>...eilzeit Praktikum/Werkstudium München Warum The Mobility House? Mit...</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://www.bayernlb.de/internet/de/blb/resp/karriere_1/studenten_und_berufseinsteiger/traineeprogramm/trainees_2024.jsp</t>
+          <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2701912/werkstudent-mwd-kreditorenbuchhaltung</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1062,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Werkstudent (m/w/d) Kreditorenbuchhaltung Praktikum/Werkstudium München</t>
+          <t>Werkstudent:in Projektmanagement Ladeinfrastruktur (m/w/d) Praktikum/Werkstudium München</t>
         </is>
       </c>
       <c r="D18" t="n">
@@ -1080,19 +1075,24 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2701912/werkstudent-mwd-kreditorenbuchhaltung</t>
+          <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2717018/werkstudentin-projektmanagement-ladeinfrastruktur-mwd</t>
         </is>
       </c>
     </row>
     <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2024-12-18</t>
+        </is>
+      </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>The Mobility House</t>
+          <t>Planet A Foods</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Werkstudent:in Projektmanagement Ladeinfrastruktur (m/w/d) Praktikum/Werkstudium München</t>
+          <t>Marketing Praktikant:in (f/m/d)</t>
         </is>
       </c>
       <c r="D19" t="n">
@@ -1100,42 +1100,38 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>...eilzeit Praktikum/Werkstudium München Warum The Mobility House? Mit...</t>
+          <t>Munich</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://www.mobilityhouse.com/de_de/unser-unternehmen/karriere/2717018/werkstudentin-projektmanagement-ladeinfrastruktur-mwd</t>
+          <t>https://planetafoods.jobs.personio.de/job/1881523</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>2024-12-18</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>Planet A Foods</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>Marketing Praktikant:in (f/m/d)</t>
-        </is>
-      </c>
-      <c r="D20" t="n">
+      <c r="A20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Munich Re</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Intern</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>Munich</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>https://planetafoods.jobs.personio.de/job/1881523</t>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>...dern Insurance Group, Inc., a Munich Re company, is a widely recog...</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>https://careers.munichre.com/en/job/amelia/intern/3342/43619098368</t>
         </is>
       </c>
     </row>
@@ -1350,26 +1346,25 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr"/>
-      <c r="B29" s="3" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>Munich Re</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>2026 Fall Intern</t>
         </is>
       </c>
-      <c r="D29" s="3" t="n">
+      <c r="D29" t="n">
         <v>1</v>
       </c>
-      <c r="E29" s="3" t="inlineStr">
+      <c r="E29" t="inlineStr">
         <is>
           <t>...dern Insurance Group, Inc., a Munich Re company, is a widely recog...</t>
         </is>
       </c>
-      <c r="F29" s="3" t="inlineStr">
+      <c r="F29" t="inlineStr">
         <is>
           <t>https://careers.munichre.com/en/job/amelia/2026-fall-intern/3342/43229230208</t>
         </is>

</xml_diff>